<commit_message>
[IMP] new control for payments
</commit_message>
<xml_diff>
--- a/payment_jetcheckout_system/static/src/xlsx/template_item_import.xlsx
+++ b/payment_jetcheckout_system/static/src/xlsx/template_item_import.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve">Partner Name</t>
   </si>
@@ -56,6 +56,15 @@
   </si>
   <si>
     <t xml:space="preserve">Sales Representative Mobile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank IBAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank Holder Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank Merchant Name</t>
   </si>
   <si>
     <t xml:space="preserve">Test Partner</t>
@@ -158,19 +167,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -363,80 +372,92 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="26.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="26.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="27.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="11.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="26.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="26.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="27.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="18.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="21.6"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="2" t="n">
+      <c r="A2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="3" t="n">
         <v>1234567890</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="2"/>
+        <v>16</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="3"/>
       <c r="F2" s="4" t="n">
         <v>5000</v>
       </c>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2" t="s">
-        <v>15</v>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>